<commit_message>
Fix oscillating torque reset and k_factor, add 3 new standard display columns
</commit_message>
<xml_diff>
--- a/summary/summary report.xlsx
+++ b/summary/summary report.xlsx
@@ -125,11 +125,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:T7" headerRowCount="1">
-  <autoFilter ref="A1:T7"/>
-  <tableColumns count="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:W13" headerRowCount="1">
+  <autoFilter ref="A1:W13"/>
+  <tableColumns count="23">
     <tableColumn id="1" name="Saved At"/>
-    <tableColumn id="2" name="Date"/>
+    <tableColumn id="2" name="Machine"/>
     <tableColumn id="3" name="Test Item"/>
     <tableColumn id="4" name="Part Name"/>
     <tableColumn id="5" name="Part No"/>
@@ -143,11 +143,14 @@
     <tableColumn id="13" name="Average Nm"/>
     <tableColumn id="14" name="Min Nm"/>
     <tableColumn id="15" name="Max Nm"/>
-    <tableColumn id="16" name="Judgment"/>
-    <tableColumn id="17" name="Remark"/>
-    <tableColumn id="18" name="Filename"/>
-    <tableColumn id="19" name="Raw CSV"/>
-    <tableColumn id="20" name="CTR Report"/>
+    <tableColumn id="16" name="Internal spec Min"/>
+    <tableColumn id="17" name="Internal spec Max"/>
+    <tableColumn id="18" name="Judgment (Drawing spec)"/>
+    <tableColumn id="19" name="Judgment (Internal spec)"/>
+    <tableColumn id="20" name="Remark"/>
+    <tableColumn id="21" name="Filename"/>
+    <tableColumn id="22" name="Raw CSV"/>
+    <tableColumn id="23" name="CTR Report"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -442,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -460,11 +463,14 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,7 +481,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Machine</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -545,25 +551,40 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Judgment</t>
+          <t>Internal spec Min</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
+          <t>Internal spec Max</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Judgment (Drawing spec)</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Judgment (Internal spec)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
           <t>Remark</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Filename</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Raw CSV</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>CTR Report</t>
         </is>
@@ -575,11 +596,6 @@
           <t>2026-06-22 16:12:07</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -617,22 +633,22 @@
       <c r="O2" t="n">
         <v>8.882244</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>260622-B-PARTNO-S-PM-01-04.csv</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260622-B-PARTNO-S-PM-01-04.csv</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260622-B-PARTNO-S-PM-01-04.xlsx</t>
         </is>
@@ -644,11 +660,6 @@
           <t>2026-06-23 13:30:59</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -686,22 +697,22 @@
       <c r="O3" t="n">
         <v>0.010935</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>260623-B-PARTNO-S-PM-01.csv</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-S-PM-01.csv</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-S-PM-01.xlsx</t>
         </is>
@@ -713,11 +724,6 @@
           <t>2026-06-23 13:31:04</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -755,22 +761,22 @@
       <c r="O4" t="n">
         <v>0.010935</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>260623-B-PARTNO-S-PM-01.csv</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-S-PM-01.csv</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-S-PM-01.xlsx</t>
         </is>
@@ -782,11 +788,6 @@
           <t>2026-06-23 13:31:08</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -824,22 +825,22 @@
       <c r="O5" t="n">
         <v>0.010935</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>260623-B-PARTNO-S-PM-01.csv</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-S-PM-01.csv</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-S-PM-01.xlsx</t>
         </is>
@@ -851,11 +852,6 @@
           <t>2026-06-23 13:37:40</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -893,22 +889,22 @@
       <c r="O6" t="n">
         <v>0.010935</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>260623-B-PARTNO-D-PM-01-01.csv</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-D-PM-01-01.csv</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-D-PM-01-01.xlsx</t>
         </is>
@@ -920,11 +916,6 @@
           <t>2026-06-23 13:37:43</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>Breakaway Torque</t>
@@ -935,7 +926,6 @@
           <t>Inner Tie Rod</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>1</v>
       </c>
@@ -954,7 +944,6 @@
           <t>S/Link #1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
         <v>-29.999996</v>
       </c>
@@ -964,25 +953,555 @@
       <c r="O7" t="n">
         <v>0.010935</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>260623-B-PARTNO-D-PM-01-02.csv</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-D-PM-01-02.csv</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-D-PM-01-02.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-11 15:47:42</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>QQ</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ITR #2</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>QQ</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>260811-B-QQ-S-PM-01-01.csv</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260811-B-QQ-S-PM-01-01.csv</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260811-B-QQ-S-PM-01-01.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-11 16:03:34</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>QQ</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ITR #2</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>QQ</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>260811-B-QQ-S-PM-01-02.csv</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260811-B-QQ-S-PM-01-02.csv</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260811-B-QQ-S-PM-01-02.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:49:07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gfgfgf</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Outer Tie Rod</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>First (F)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ITR #2</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>12</v>
+      </c>
+      <c r="O10" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>12</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>260813-B-EW-F-PM-01-01.csv</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260813-B-EW-F-PM-01-01.csv</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260813-B-EW-F-PM-01-01.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-13 09:05:54</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>gfgfgf</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Outer Tie Rod</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>First (F)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ITR #2</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>12</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>12</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>260813-B-EW-F-PM-01-02.csv</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260813-B-EW-F-PM-01-02.csv</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260813-B-EW-F-PM-01-02.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-13 09:11:20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>gfgfgf</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Outer Tie Rod</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>First (F)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>ITR #2</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>12</v>
+      </c>
+      <c r="O12" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>12</v>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>260813-B-EW-F-PM-01-03.csv</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260813-B-EW-F-PM-01-03.csv</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260813-B-EW-F-PM-01-03.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-13 09:15:51</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>gfgfgf</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Outer Tie Rod</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>EW</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>First (F)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ITR #2</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>12</v>
+      </c>
+      <c r="O13" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>12</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>260813-B-EW-F-PM-01-04.csv</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260813-B-EW-F-PM-01-04.csv</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260813-B-EW-F-PM-01-04.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>